<commit_message>
Corrige nome do Presidente e presenca de Ruy Sandes Leal Junior em 28/07
</commit_message>
<xml_diff>
--- a/Rotary_Frequencia_Mestre.xlsx
+++ b/Rotary_Frequencia_Mestre.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="94">
   <si>
     <t xml:space="preserve">Nº</t>
   </si>
@@ -98,7 +98,7 @@
     <t xml:space="preserve">Alexandre Tarquínio Lara Medrado</t>
   </si>
   <si>
-    <t xml:space="preserve">Bruno Nunes Silva</t>
+    <t xml:space="preserve">Bruno de Nunes Silva</t>
   </si>
   <si>
     <t xml:space="preserve">Carlos Olimpio Ferraz Ribeiro Junior</t>
@@ -290,7 +290,19 @@
     <t xml:space="preserve">Diretoria (exibida no site)</t>
   </si>
   <si>
-    <t xml:space="preserve">Presidente: Bruno Nunes Silva. 1º Secretário: José Carlos Rodrigues.</t>
+    <t xml:space="preserve">Presidente: Bruno de Nunes Silva. 1º Secretário: José Carlos Rodrigues.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bruno de Nunes Silva (linha 9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome corrigido de 'Bruno Nunes Silva' para 'Bruno de Nunes Silva' (grafia correta) em 18/08/2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ruy Sandes Leal Junior (linha 49)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrigido de falta (A) para presente (P) em 28/07 — confirmado pelo Jefferson em 18/08/2026 que ele esteve na reunião.</t>
   </si>
 </sst>
 </file>
@@ -2559,15 +2571,15 @@
         <v>36</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H48" s="2" t="n">
         <f aca="false">COUNTIF(D48:G48,"P")+COUNTIF(D48:G48,"AJ")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I48" s="2" t="n">
         <f aca="false">COUNTIF(D48:G48,"A")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J48" s="2" t="n">
         <f aca="false">4-COUNTIF(D48:G48,"-")</f>
@@ -2575,7 +2587,7 @@
       </c>
       <c r="K48" s="4" t="n">
         <f aca="false">IF(J48=0,"-",H48/J48)</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="L48" s="3"/>
     </row>
@@ -2715,7 +2727,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -2822,6 +2834,22 @@
       </c>
       <c r="B14" s="7" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>